<commit_message>
Corrigir cálculo da média mensal: ÷12 anos completos, ÷meses corridos ano atual
https://claude.ai/code/session_01SyvqAv69ozhh5ptHC31e4L
</commit_message>
<xml_diff>
--- a/relatorio_grao_por_vendedor.xlsx
+++ b/relatorio_grao_por_vendedor.xlsx
@@ -527,10 +527,10 @@
         <v>24</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>4</v>
+        <v>0.3</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>24</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3">
@@ -562,10 +562,10 @@
         <v>528</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>44</v>
+        <v>7.3</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>264</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>6</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
@@ -632,10 +632,10 @@
         <v>6</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -667,10 +667,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
@@ -737,10 +737,10 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9">
@@ -807,10 +807,10 @@
         <v>66</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="11">
@@ -842,10 +842,10 @@
         <v>6</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="12">
@@ -1157,10 +1157,10 @@
         <v>72</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>7.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1227,10 +1227,10 @@
         <v>126</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>11.4</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="23">
@@ -1332,10 +1332,10 @@
         <v>48</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="26">
@@ -1367,10 +1367,10 @@
         <v>66</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="27">
@@ -1402,10 +1402,10 @@
         <v>24</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="28">
@@ -1437,10 +1437,10 @@
         <v>102</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>14.4</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="29">
@@ -1507,10 +1507,10 @@
         <v>60</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>15</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="31">
@@ -1542,10 +1542,10 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="32">
@@ -1577,10 +1577,10 @@
         <v>180</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">
@@ -1647,10 +1647,10 @@
         <v>168</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>4</v>
+        <v>2.3</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>24</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="35">
@@ -1752,10 +1752,10 @@
         <v>84</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="38">
@@ -1892,10 +1892,10 @@
         <v>306</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>38.4</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="42">
@@ -1927,10 +1927,10 @@
         <v>150</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>30</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="43">
@@ -1962,10 +1962,10 @@
         <v>300</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>30</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="44">
@@ -1997,10 +1997,10 @@
         <v>120</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>24</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="45">
@@ -2172,10 +2172,10 @@
         <v>366</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>6.8</v>
+        <v>5.1</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>40.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="50">
@@ -2312,10 +2312,10 @@
         <v>84</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="54">
@@ -2382,10 +2382,10 @@
         <v>1278</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>21.3</v>
+        <v>17.8</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>127.8</v>
+        <v>106.8</v>
       </c>
     </row>
     <row r="56">
@@ -2417,10 +2417,10 @@
         <v>510</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>21.2</v>
+        <v>14.2</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>127.2</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="57">
@@ -2452,10 +2452,10 @@
         <v>6</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="58">
@@ -2557,10 +2557,10 @@
         <v>120</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>4</v>
+        <v>1.7</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>24</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="61">
@@ -2627,10 +2627,10 @@
         <v>372</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>6.2</v>
+        <v>5.2</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>37.2</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="63">
@@ -2662,10 +2662,10 @@
         <v>54</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>6.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="64">
@@ -2697,10 +2697,10 @@
         <v>12</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="65">
@@ -2732,10 +2732,10 @@
         <v>12</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="66">
@@ -2767,10 +2767,10 @@
         <v>24</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="67">
@@ -2802,10 +2802,10 @@
         <v>420</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>35</v>
+        <v>5.8</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>210</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="68">
@@ -2942,10 +2942,10 @@
         <v>24</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="72">
@@ -2977,10 +2977,10 @@
         <v>12</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="73">
@@ -3082,10 +3082,10 @@
         <v>66</v>
       </c>
       <c r="H75" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I75" s="4" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="76">
@@ -3117,10 +3117,10 @@
         <v>30</v>
       </c>
       <c r="H76" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I76" s="4" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="77">
@@ -3152,10 +3152,10 @@
         <v>48</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="78">
@@ -3187,10 +3187,10 @@
         <v>12</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="79">
@@ -3327,10 +3327,10 @@
         <v>54</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -3362,10 +3362,10 @@
         <v>48</v>
       </c>
       <c r="H83" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I83" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="84">
@@ -3397,10 +3397,10 @@
         <v>24</v>
       </c>
       <c r="H84" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I84" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="85">
@@ -3432,10 +3432,10 @@
         <v>48</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>6.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="86">
@@ -3467,10 +3467,10 @@
         <v>24</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="87">
@@ -3642,10 +3642,10 @@
         <v>42</v>
       </c>
       <c r="H91" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I91" s="4" t="n">
-        <v>6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="92">
@@ -3677,10 +3677,10 @@
         <v>18</v>
       </c>
       <c r="H92" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I92" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
@@ -3712,10 +3712,10 @@
         <v>54</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="94">
@@ -3747,10 +3747,10 @@
         <v>30</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I94" s="3" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="95">
@@ -3817,10 +3817,10 @@
         <v>72</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>14.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97">
@@ -3852,10 +3852,10 @@
         <v>72</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I97" s="3" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="98">
@@ -3992,10 +3992,10 @@
         <v>114</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="I101" s="3" t="n">
-        <v>11.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="102">
@@ -4062,10 +4062,10 @@
         <v>66</v>
       </c>
       <c r="H103" s="4" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I103" s="4" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="104">
@@ -4097,10 +4097,10 @@
         <v>18</v>
       </c>
       <c r="H104" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I104" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
@@ -4132,10 +4132,10 @@
         <v>168</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="I105" s="3" t="n">
-        <v>16.8</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="106">
@@ -4167,10 +4167,10 @@
         <v>72</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="I106" s="3" t="n">
-        <v>14.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107">
@@ -4202,10 +4202,10 @@
         <v>18</v>
       </c>
       <c r="H107" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I107" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="108">
@@ -4237,10 +4237,10 @@
         <v>6</v>
       </c>
       <c r="H108" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I108" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="109">
@@ -4307,10 +4307,10 @@
         <v>234</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>7.8</v>
+        <v>6.5</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>46.8</v>
+        <v>39</v>
       </c>
     </row>
     <row r="111">
@@ -4377,10 +4377,10 @@
         <v>6</v>
       </c>
       <c r="H112" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I112" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="113">
@@ -4412,10 +4412,10 @@
         <v>30</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="I113" s="3" t="n">
-        <v>10.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="114">
@@ -4447,10 +4447,10 @@
         <v>252</v>
       </c>
       <c r="H114" s="4" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="I114" s="4" t="n">
-        <v>22.8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="115">
@@ -4587,10 +4587,10 @@
         <v>18</v>
       </c>
       <c r="H118" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I118" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="119">
@@ -4797,10 +4797,10 @@
         <v>42</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I124" s="3" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="125">
@@ -4832,10 +4832,10 @@
         <v>54</v>
       </c>
       <c r="H125" s="4" t="n">
-        <v>4.5</v>
+        <v>0.8</v>
       </c>
       <c r="I125" s="4" t="n">
-        <v>27</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="126">
@@ -4867,10 +4867,10 @@
         <v>90</v>
       </c>
       <c r="H126" s="4" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I126" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="127">
@@ -4937,10 +4937,10 @@
         <v>12</v>
       </c>
       <c r="H128" s="4" t="n">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="I128" s="4" t="n">
-        <v>12</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="129">
@@ -4972,10 +4972,10 @@
         <v>18</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="I129" s="3" t="n">
-        <v>18</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="130">
@@ -5007,10 +5007,10 @@
         <v>96</v>
       </c>
       <c r="H130" s="4" t="n">
-        <v>2.3</v>
+        <v>1.3</v>
       </c>
       <c r="I130" s="4" t="n">
-        <v>13.8</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="131">
@@ -5112,10 +5112,10 @@
         <v>198</v>
       </c>
       <c r="H133" s="4" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="I133" s="4" t="n">
-        <v>18</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="134">
@@ -5217,10 +5217,10 @@
         <v>60</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="I136" s="3" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="137">
@@ -5252,10 +5252,10 @@
         <v>54</v>
       </c>
       <c r="H137" s="4" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="I137" s="4" t="n">
-        <v>6.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="138">
@@ -5287,10 +5287,10 @@
         <v>24</v>
       </c>
       <c r="H138" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I138" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="139">
@@ -5322,10 +5322,10 @@
         <v>30</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I139" s="3" t="n">
-        <v>6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="140">
@@ -5357,10 +5357,10 @@
         <v>12</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I140" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="141">
@@ -5392,10 +5392,10 @@
         <v>6</v>
       </c>
       <c r="H141" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I141" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="142">
@@ -5427,10 +5427,10 @@
         <v>48</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I142" s="3" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="143">
@@ -5462,10 +5462,10 @@
         <v>18</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I143" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="144">
@@ -5497,10 +5497,10 @@
         <v>54</v>
       </c>
       <c r="H144" s="4" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="I144" s="4" t="n">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="145">
@@ -5567,10 +5567,10 @@
         <v>6</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I146" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="147">
@@ -5602,10 +5602,10 @@
         <v>42</v>
       </c>
       <c r="H147" s="4" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="I147" s="4" t="n">
-        <v>7.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="148">
@@ -5637,10 +5637,10 @@
         <v>24</v>
       </c>
       <c r="H148" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I148" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="149">
@@ -5672,10 +5672,10 @@
         <v>12</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="150">
@@ -5707,10 +5707,10 @@
         <v>30</v>
       </c>
       <c r="H150" s="4" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="I150" s="4" t="n">
-        <v>10.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="151">
@@ -5742,10 +5742,10 @@
         <v>6</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I151" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="152">
@@ -5777,10 +5777,10 @@
         <v>24</v>
       </c>
       <c r="H152" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I152" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="153">
@@ -5812,10 +5812,10 @@
         <v>18</v>
       </c>
       <c r="H153" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I153" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154">
@@ -5847,10 +5847,10 @@
         <v>24</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="I154" s="3" t="n">
-        <v>7.8</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="155">
@@ -5882,10 +5882,10 @@
         <v>6</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I155" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="156">
@@ -5917,10 +5917,10 @@
         <v>48</v>
       </c>
       <c r="H156" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I156" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="157">
@@ -5952,10 +5952,10 @@
         <v>18</v>
       </c>
       <c r="H157" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I157" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="158">
@@ -5987,10 +5987,10 @@
         <v>12</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I158" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="159">
@@ -6022,10 +6022,10 @@
         <v>24</v>
       </c>
       <c r="H159" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I159" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="160">
@@ -6057,10 +6057,10 @@
         <v>12</v>
       </c>
       <c r="H160" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I160" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="161">
@@ -6127,10 +6127,10 @@
         <v>66</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="I162" s="3" t="n">
-        <v>13.2</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="163">
@@ -6162,10 +6162,10 @@
         <v>24</v>
       </c>
       <c r="H163" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I163" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="164">
@@ -6197,10 +6197,10 @@
         <v>12</v>
       </c>
       <c r="H164" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I164" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="165">
@@ -6267,10 +6267,10 @@
         <v>24</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I166" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="167">
@@ -6302,10 +6302,10 @@
         <v>30</v>
       </c>
       <c r="H167" s="4" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="I167" s="4" t="n">
-        <v>10.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="168">
@@ -6337,10 +6337,10 @@
         <v>18</v>
       </c>
       <c r="H168" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I168" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169">
@@ -6442,10 +6442,10 @@
         <v>54</v>
       </c>
       <c r="H171" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I171" s="4" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="172">
@@ -6477,10 +6477,10 @@
         <v>18</v>
       </c>
       <c r="H172" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I172" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173">
@@ -6687,10 +6687,10 @@
         <v>30</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I178" s="3" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="179">
@@ -6722,10 +6722,10 @@
         <v>156</v>
       </c>
       <c r="H179" s="4" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="I179" s="4" t="n">
-        <v>15.6</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="180">
@@ -6757,10 +6757,10 @@
         <v>54</v>
       </c>
       <c r="H180" s="4" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="I180" s="4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181">
@@ -6932,10 +6932,10 @@
         <v>90</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="I185" s="3" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="186">
@@ -6967,10 +6967,10 @@
         <v>24</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I186" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="187">
@@ -7002,10 +7002,10 @@
         <v>60</v>
       </c>
       <c r="H187" s="4" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="I187" s="4" t="n">
-        <v>19.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="188">
@@ -7037,10 +7037,10 @@
         <v>24</v>
       </c>
       <c r="H188" s="4" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I188" s="4" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="189">
@@ -7072,10 +7072,10 @@
         <v>60</v>
       </c>
       <c r="H189" s="4" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="I189" s="4" t="n">
-        <v>15</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="190">
@@ -7107,10 +7107,10 @@
         <v>66</v>
       </c>
       <c r="H190" s="3" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="I190" s="3" t="n">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="191">
@@ -7142,10 +7142,10 @@
         <v>24</v>
       </c>
       <c r="H191" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I191" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="192">
@@ -7177,10 +7177,10 @@
         <v>6</v>
       </c>
       <c r="H192" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I192" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="193">
@@ -7212,10 +7212,10 @@
         <v>30</v>
       </c>
       <c r="H193" s="4" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="I193" s="4" t="n">
-        <v>7.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="194">
@@ -7387,10 +7387,10 @@
         <v>48</v>
       </c>
       <c r="H198" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I198" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="199">
@@ -7422,10 +7422,10 @@
         <v>18</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I199" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="200">
@@ -7457,10 +7457,10 @@
         <v>48</v>
       </c>
       <c r="H200" s="4" t="n">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="I200" s="4" t="n">
-        <v>12</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="201">
@@ -7492,10 +7492,10 @@
         <v>24</v>
       </c>
       <c r="H201" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I201" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="202">
@@ -7527,10 +7527,10 @@
         <v>18</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I202" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="203">
@@ -7562,10 +7562,10 @@
         <v>12</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I203" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="204">
@@ -7702,10 +7702,10 @@
         <v>180</v>
       </c>
       <c r="H207" s="4" t="n">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="I207" s="4" t="n">
-        <v>22.8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="208">
@@ -7737,10 +7737,10 @@
         <v>54</v>
       </c>
       <c r="H208" s="4" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="I208" s="4" t="n">
-        <v>13.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="209">
@@ -7842,10 +7842,10 @@
         <v>42</v>
       </c>
       <c r="H211" s="4" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="I211" s="4" t="n">
-        <v>10.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="212">
@@ -7877,10 +7877,10 @@
         <v>24</v>
       </c>
       <c r="H212" s="4" t="n">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="I212" s="4" t="n">
-        <v>12</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="213">
@@ -7912,10 +7912,10 @@
         <v>24</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I213" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="214">
@@ -7947,10 +7947,10 @@
         <v>180</v>
       </c>
       <c r="H214" s="4" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="I214" s="4" t="n">
-        <v>19.8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="215">
@@ -8052,10 +8052,10 @@
         <v>66</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="I217" s="3" t="n">
-        <v>13.2</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="218">
@@ -8192,10 +8192,10 @@
         <v>48</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="I221" s="3" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="222">
@@ -8297,10 +8297,10 @@
         <v>348</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>29</v>
+        <v>4.8</v>
       </c>
       <c r="I224" s="3" t="n">
-        <v>174</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="225">
@@ -8332,10 +8332,10 @@
         <v>48</v>
       </c>
       <c r="H225" s="4" t="n">
-        <v>4</v>
+        <v>0.7</v>
       </c>
       <c r="I225" s="4" t="n">
-        <v>24</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="226">
@@ -8367,10 +8367,10 @@
         <v>270</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>5.6</v>
+        <v>3.8</v>
       </c>
       <c r="I226" s="3" t="n">
-        <v>33.6</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="227">
@@ -8402,10 +8402,10 @@
         <v>150</v>
       </c>
       <c r="H227" s="3" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="I227" s="3" t="n">
-        <v>30</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="228">
@@ -8437,10 +8437,10 @@
         <v>324</v>
       </c>
       <c r="H228" s="4" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="I228" s="4" t="n">
-        <v>29.4</v>
+        <v>27</v>
       </c>
     </row>
     <row r="229">
@@ -8507,10 +8507,10 @@
         <v>168</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="I230" s="3" t="n">
-        <v>16.8</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="231">
@@ -8647,10 +8647,10 @@
         <v>120</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>5</v>
+        <v>1.7</v>
       </c>
       <c r="I234" s="3" t="n">
-        <v>30</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="235">
@@ -8682,10 +8682,10 @@
         <v>60</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>5</v>
+        <v>1.7</v>
       </c>
       <c r="I235" s="3" t="n">
-        <v>30</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="236">
@@ -8787,10 +8787,10 @@
         <v>162</v>
       </c>
       <c r="H238" s="3" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="I238" s="3" t="n">
-        <v>15</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="239">
@@ -8822,10 +8822,10 @@
         <v>72</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="I239" s="3" t="n">
-        <v>14.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="240">
@@ -8857,10 +8857,10 @@
         <v>258</v>
       </c>
       <c r="H240" s="4" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="I240" s="4" t="n">
-        <v>28.8</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="241">
@@ -8927,10 +8927,10 @@
         <v>264</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>6.3</v>
+        <v>3.7</v>
       </c>
       <c r="I242" s="3" t="n">
-        <v>37.8</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="243">
@@ -8997,10 +8997,10 @@
         <v>600</v>
       </c>
       <c r="H244" s="4" t="n">
-        <v>25</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I244" s="4" t="n">
-        <v>150</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="245">
@@ -9032,10 +9032,10 @@
         <v>150</v>
       </c>
       <c r="H245" s="4" t="n">
-        <v>25</v>
+        <v>4.2</v>
       </c>
       <c r="I245" s="4" t="n">
-        <v>150</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="246">
@@ -9067,10 +9067,10 @@
         <v>12</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I246" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="247">
@@ -9102,10 +9102,10 @@
         <v>30</v>
       </c>
       <c r="H247" s="4" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="I247" s="4" t="n">
-        <v>6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="248">
@@ -9137,10 +9137,10 @@
         <v>84</v>
       </c>
       <c r="H248" s="3" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="I248" s="3" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="249">
@@ -9172,10 +9172,10 @@
         <v>12</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I249" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="250">
@@ -9207,10 +9207,10 @@
         <v>18</v>
       </c>
       <c r="H250" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I250" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="251">
@@ -9242,10 +9242,10 @@
         <v>6</v>
       </c>
       <c r="H251" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I251" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="252">
@@ -9277,10 +9277,10 @@
         <v>438</v>
       </c>
       <c r="H252" s="3" t="n">
-        <v>7.3</v>
+        <v>6.1</v>
       </c>
       <c r="I252" s="3" t="n">
-        <v>43.8</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="253">
@@ -9347,10 +9347,10 @@
         <v>96</v>
       </c>
       <c r="H254" s="4" t="n">
-        <v>2.3</v>
+        <v>1.3</v>
       </c>
       <c r="I254" s="4" t="n">
-        <v>13.8</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="255">
@@ -9382,10 +9382,10 @@
         <v>24</v>
       </c>
       <c r="H255" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I255" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="256">
@@ -9417,10 +9417,10 @@
         <v>180</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="I256" s="3" t="n">
-        <v>16.2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="257">
@@ -9452,10 +9452,10 @@
         <v>90</v>
       </c>
       <c r="H257" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I257" s="3" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="258">
@@ -9487,10 +9487,10 @@
         <v>84</v>
       </c>
       <c r="H258" s="4" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="I258" s="4" t="n">
-        <v>10.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="259">
@@ -9522,10 +9522,10 @@
         <v>36</v>
       </c>
       <c r="H259" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I259" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="260">
@@ -9557,10 +9557,10 @@
         <v>24</v>
       </c>
       <c r="H260" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I260" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="261">
@@ -9592,10 +9592,10 @@
         <v>12</v>
       </c>
       <c r="H261" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I261" s="4" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="262">
@@ -9627,10 +9627,10 @@
         <v>12</v>
       </c>
       <c r="H262" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I262" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="263">
@@ -9662,10 +9662,10 @@
         <v>30</v>
       </c>
       <c r="H263" s="3" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="I263" s="3" t="n">
-        <v>7.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="264">
@@ -9697,10 +9697,10 @@
         <v>24</v>
       </c>
       <c r="H264" s="3" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I264" s="3" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="265">
@@ -9732,10 +9732,10 @@
         <v>66</v>
       </c>
       <c r="H265" s="4" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="I265" s="4" t="n">
-        <v>10.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="266">
@@ -9837,10 +9837,10 @@
         <v>42</v>
       </c>
       <c r="H268" s="3" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I268" s="3" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="269">
@@ -9872,10 +9872,10 @@
         <v>30</v>
       </c>
       <c r="H269" s="4" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I269" s="4" t="n">
-        <v>7.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="270">
@@ -9907,10 +9907,10 @@
         <v>24</v>
       </c>
       <c r="H270" s="3" t="n">
-        <v>4</v>
+        <v>0.7</v>
       </c>
       <c r="I270" s="3" t="n">
-        <v>24</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="271">
@@ -10327,10 +10327,10 @@
         <v>108</v>
       </c>
       <c r="H282" s="4" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="I282" s="4" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="283">
@@ -10362,10 +10362,10 @@
         <v>48</v>
       </c>
       <c r="H283" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I283" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="284">
@@ -10397,10 +10397,10 @@
         <v>48</v>
       </c>
       <c r="H284" s="4" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="I284" s="4" t="n">
-        <v>16.2</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="285">
@@ -10642,10 +10642,10 @@
         <v>60</v>
       </c>
       <c r="H291" s="3" t="n">
-        <v>5</v>
+        <v>1.7</v>
       </c>
       <c r="I291" s="3" t="n">
-        <v>30</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="292">
@@ -10677,10 +10677,10 @@
         <v>126</v>
       </c>
       <c r="H292" s="3" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="I292" s="3" t="n">
-        <v>25.2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="293">
@@ -10782,10 +10782,10 @@
         <v>66</v>
       </c>
       <c r="H295" s="3" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="I295" s="3" t="n">
-        <v>8.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="296">
@@ -10887,10 +10887,10 @@
         <v>150</v>
       </c>
       <c r="H298" s="3" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="I298" s="3" t="n">
-        <v>13.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="299">
@@ -10922,10 +10922,10 @@
         <v>30</v>
       </c>
       <c r="H299" s="3" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I299" s="3" t="n">
-        <v>7.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="300">
@@ -11062,10 +11062,10 @@
         <v>102</v>
       </c>
       <c r="H303" s="3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="I303" s="3" t="n">
-        <v>20.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="304">
@@ -11237,10 +11237,10 @@
         <v>312</v>
       </c>
       <c r="H308" s="4" t="n">
-        <v>5.2</v>
+        <v>4.3</v>
       </c>
       <c r="I308" s="4" t="n">
-        <v>31.2</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="309">
@@ -11377,10 +11377,10 @@
         <v>3168</v>
       </c>
       <c r="H312" s="4" t="n">
-        <v>52.8</v>
+        <v>44</v>
       </c>
       <c r="I312" s="4" t="n">
-        <v>316.8</v>
+        <v>264</v>
       </c>
     </row>
     <row r="313">
@@ -11412,10 +11412,10 @@
         <v>882</v>
       </c>
       <c r="H313" s="4" t="n">
-        <v>36.8</v>
+        <v>24.5</v>
       </c>
       <c r="I313" s="4" t="n">
-        <v>220.8</v>
+        <v>147</v>
       </c>
     </row>
     <row r="314">
@@ -11447,10 +11447,10 @@
         <v>36</v>
       </c>
       <c r="H314" s="3" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="I314" s="3" t="n">
-        <v>7.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="315">
@@ -11517,10 +11517,10 @@
         <v>132</v>
       </c>
       <c r="H316" s="4" t="n">
-        <v>4.4</v>
+        <v>3.7</v>
       </c>
       <c r="I316" s="4" t="n">
-        <v>26.4</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="317">
@@ -11587,10 +11587,10 @@
         <v>36</v>
       </c>
       <c r="H318" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I318" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="319">
@@ -11762,10 +11762,10 @@
         <v>90</v>
       </c>
       <c r="H323" s="4" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="I323" s="4" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="324">
@@ -11797,10 +11797,10 @@
         <v>168</v>
       </c>
       <c r="H324" s="3" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="I324" s="3" t="n">
-        <v>15</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="325">
@@ -11867,10 +11867,10 @@
         <v>108</v>
       </c>
       <c r="H326" s="4" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="I326" s="4" t="n">
-        <v>13.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="327">
@@ -11902,10 +11902,10 @@
         <v>12</v>
       </c>
       <c r="H327" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I327" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="328">
@@ -11937,10 +11937,10 @@
         <v>420</v>
       </c>
       <c r="H328" s="4" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="I328" s="4" t="n">
-        <v>52.8</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="329">
@@ -12007,10 +12007,10 @@
         <v>24</v>
       </c>
       <c r="H330" s="3" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I330" s="3" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="331">
@@ -12042,10 +12042,10 @@
         <v>30</v>
       </c>
       <c r="H331" s="3" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I331" s="3" t="n">
-        <v>7.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="332">
@@ -12077,10 +12077,10 @@
         <v>6</v>
       </c>
       <c r="H332" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I332" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="333">
@@ -12112,10 +12112,10 @@
         <v>24</v>
       </c>
       <c r="H333" s="3" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I333" s="3" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="334">
@@ -12147,10 +12147,10 @@
         <v>24</v>
       </c>
       <c r="H334" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I334" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="335">
@@ -12182,10 +12182,10 @@
         <v>24</v>
       </c>
       <c r="H335" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I335" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="336">
@@ -12217,10 +12217,10 @@
         <v>66</v>
       </c>
       <c r="H336" s="3" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="I336" s="3" t="n">
-        <v>7.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="337">
@@ -12252,10 +12252,10 @@
         <v>24</v>
       </c>
       <c r="H337" s="3" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I337" s="3" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="338">
@@ -12287,10 +12287,10 @@
         <v>60</v>
       </c>
       <c r="H338" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I338" s="4" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="339">
@@ -12322,10 +12322,10 @@
         <v>30</v>
       </c>
       <c r="H339" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I339" s="4" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="340">
@@ -12357,10 +12357,10 @@
         <v>6</v>
       </c>
       <c r="H340" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I340" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="341">
@@ -12392,10 +12392,10 @@
         <v>42</v>
       </c>
       <c r="H341" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I341" s="4" t="n">
-        <v>6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="342">
@@ -12427,10 +12427,10 @@
         <v>18</v>
       </c>
       <c r="H342" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I342" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="343">
@@ -12567,10 +12567,10 @@
         <v>42</v>
       </c>
       <c r="H346" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I346" s="4" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="347">
@@ -12742,10 +12742,10 @@
         <v>186</v>
       </c>
       <c r="H351" s="3" t="n">
-        <v>5.2</v>
+        <v>2.6</v>
       </c>
       <c r="I351" s="3" t="n">
-        <v>31.2</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="352">
@@ -12777,10 +12777,10 @@
         <v>150</v>
       </c>
       <c r="H352" s="3" t="n">
-        <v>4.2</v>
+        <v>2.1</v>
       </c>
       <c r="I352" s="3" t="n">
-        <v>25.2</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="353">
@@ -12882,10 +12882,10 @@
         <v>30</v>
       </c>
       <c r="H355" s="4" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="I355" s="4" t="n">
-        <v>15</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="356">
@@ -12987,10 +12987,10 @@
         <v>120</v>
       </c>
       <c r="H358" s="4" t="n">
-        <v>4</v>
+        <v>1.7</v>
       </c>
       <c r="I358" s="4" t="n">
-        <v>24</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="359">
@@ -13022,10 +13022,10 @@
         <v>30</v>
       </c>
       <c r="H359" s="4" t="n">
-        <v>5</v>
+        <v>0.8</v>
       </c>
       <c r="I359" s="4" t="n">
-        <v>30</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="360">
@@ -13267,10 +13267,10 @@
         <v>96</v>
       </c>
       <c r="H366" s="4" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="I366" s="4" t="n">
-        <v>12</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="367">
@@ -13372,10 +13372,10 @@
         <v>36</v>
       </c>
       <c r="H369" s="4" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="I369" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="370">
@@ -13407,10 +13407,10 @@
         <v>144</v>
       </c>
       <c r="H370" s="3" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="I370" s="3" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="371">
@@ -13477,10 +13477,10 @@
         <v>150</v>
       </c>
       <c r="H372" s="4" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="I372" s="4" t="n">
-        <v>13.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="373">
@@ -13547,10 +13547,10 @@
         <v>192</v>
       </c>
       <c r="H374" s="3" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="I374" s="3" t="n">
-        <v>17.4</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="375">
@@ -13582,10 +13582,10 @@
         <v>84</v>
       </c>
       <c r="H375" s="3" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="I375" s="3" t="n">
-        <v>16.8</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="376">
@@ -13617,10 +13617,10 @@
         <v>6</v>
       </c>
       <c r="H376" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I376" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="377">
@@ -13652,10 +13652,10 @@
         <v>234</v>
       </c>
       <c r="H377" s="3" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="I377" s="3" t="n">
-        <v>21</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="378">
@@ -13722,10 +13722,10 @@
         <v>90</v>
       </c>
       <c r="H379" s="4" t="n">
-        <v>2.5</v>
+        <v>1.2</v>
       </c>
       <c r="I379" s="4" t="n">
-        <v>15</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="380">
@@ -13757,10 +13757,10 @@
         <v>330</v>
       </c>
       <c r="H380" s="3" t="n">
-        <v>6.1</v>
+        <v>4.6</v>
       </c>
       <c r="I380" s="3" t="n">
-        <v>36.6</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="381">
@@ -13792,10 +13792,10 @@
         <v>150</v>
       </c>
       <c r="H381" s="3" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="I381" s="3" t="n">
-        <v>30</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="382">
@@ -13827,10 +13827,10 @@
         <v>618</v>
       </c>
       <c r="H382" s="4" t="n">
-        <v>10.3</v>
+        <v>8.6</v>
       </c>
       <c r="I382" s="4" t="n">
-        <v>61.8</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="383">
@@ -13862,10 +13862,10 @@
         <v>204</v>
       </c>
       <c r="H383" s="4" t="n">
-        <v>6.8</v>
+        <v>5.7</v>
       </c>
       <c r="I383" s="4" t="n">
-        <v>40.8</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="384">
@@ -13897,10 +13897,10 @@
         <v>24</v>
       </c>
       <c r="H384" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I384" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="385">
@@ -13967,10 +13967,10 @@
         <v>54</v>
       </c>
       <c r="H386" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="I386" s="4" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="387">
@@ -14037,10 +14037,10 @@
         <v>102</v>
       </c>
       <c r="H388" s="3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="I388" s="3" t="n">
-        <v>20.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="389">
@@ -14072,10 +14072,10 @@
         <v>66</v>
       </c>
       <c r="H389" s="4" t="n">
-        <v>2.2</v>
+        <v>0.9</v>
       </c>
       <c r="I389" s="4" t="n">
-        <v>13.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="390">
@@ -14142,10 +14142,10 @@
         <v>72</v>
       </c>
       <c r="H391" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I391" s="3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="392">
@@ -14247,10 +14247,10 @@
         <v>6</v>
       </c>
       <c r="H394" s="3" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I394" s="3" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="395">
@@ -14282,10 +14282,10 @@
         <v>96</v>
       </c>
       <c r="H395" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="I395" s="4" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="396">
@@ -14317,10 +14317,10 @@
         <v>6</v>
       </c>
       <c r="H396" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I396" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="397">
@@ -14352,10 +14352,10 @@
         <v>84</v>
       </c>
       <c r="H397" s="3" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="I397" s="3" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="398">
@@ -14387,10 +14387,10 @@
         <v>42</v>
       </c>
       <c r="H398" s="3" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I398" s="3" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="399">
@@ -14422,10 +14422,10 @@
         <v>24</v>
       </c>
       <c r="H399" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I399" s="4" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="400">
@@ -14457,10 +14457,10 @@
         <v>30</v>
       </c>
       <c r="H400" s="3" t="n">
-        <v>5</v>
+        <v>0.4</v>
       </c>
       <c r="I400" s="3" t="n">
-        <v>30</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="401">
@@ -14492,10 +14492,10 @@
         <v>78</v>
       </c>
       <c r="H401" s="4" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="I401" s="4" t="n">
-        <v>11.4</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="402">
@@ -14562,10 +14562,10 @@
         <v>12</v>
       </c>
       <c r="H403" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I403" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="404">
@@ -14597,10 +14597,10 @@
         <v>18</v>
       </c>
       <c r="H404" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I404" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="405">
@@ -14667,10 +14667,10 @@
         <v>102</v>
       </c>
       <c r="H406" s="3" t="n">
-        <v>5.7</v>
+        <v>2.8</v>
       </c>
       <c r="I406" s="3" t="n">
-        <v>34.2</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="407">
@@ -14702,10 +14702,10 @@
         <v>12</v>
       </c>
       <c r="H407" s="4" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I407" s="4" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="408">
@@ -14737,10 +14737,10 @@
         <v>18</v>
       </c>
       <c r="H408" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I408" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="I408" s="3" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="409">
@@ -14772,10 +14772,10 @@
         <v>18</v>
       </c>
       <c r="H409" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="I409" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="410">
@@ -14807,10 +14807,10 @@
         <v>6</v>
       </c>
       <c r="H410" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I410" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="411">
@@ -14842,10 +14842,10 @@
         <v>90</v>
       </c>
       <c r="H411" s="3" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="I411" s="3" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="412">
@@ -14877,10 +14877,10 @@
         <v>30</v>
       </c>
       <c r="H412" s="3" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I412" s="3" t="n">
-        <v>7.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="413">
@@ -14947,10 +14947,10 @@
         <v>48</v>
       </c>
       <c r="H414" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="I414" s="4" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="415">
@@ -15122,10 +15122,10 @@
         <v>84</v>
       </c>
       <c r="H419" s="3" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="I419" s="3" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="420">
@@ -15157,10 +15157,10 @@
         <v>30</v>
       </c>
       <c r="H420" s="3" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I420" s="3" t="n">
-        <v>7.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="421">
@@ -15192,10 +15192,10 @@
         <v>72</v>
       </c>
       <c r="H421" s="4" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="I421" s="4" t="n">
-        <v>7.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="422">
@@ -15262,10 +15262,10 @@
         <v>30</v>
       </c>
       <c r="H423" s="3" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="I423" s="3" t="n">
-        <v>10.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="424">
@@ -15297,10 +15297,10 @@
         <v>66</v>
       </c>
       <c r="H424" s="3" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="I424" s="3" t="n">
-        <v>8.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="425">
@@ -15332,10 +15332,10 @@
         <v>24</v>
       </c>
       <c r="H425" s="3" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I425" s="3" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="426">
@@ -15367,10 +15367,10 @@
         <v>42</v>
       </c>
       <c r="H426" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I426" s="4" t="n">
-        <v>6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="427">
@@ -15402,10 +15402,10 @@
         <v>24</v>
       </c>
       <c r="H427" s="4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I427" s="4" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="428">
@@ -15472,10 +15472,10 @@
         <v>12</v>
       </c>
       <c r="H429" s="3" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I429" s="3" t="n">
-        <v>12</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="430">
@@ -15647,10 +15647,10 @@
         <v>72</v>
       </c>
       <c r="H434" s="4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I434" s="4" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="435">
@@ -15682,10 +15682,10 @@
         <v>30</v>
       </c>
       <c r="H435" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I435" s="4" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="436">
@@ -15752,10 +15752,10 @@
         <v>72</v>
       </c>
       <c r="H437" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="I437" s="3" t="n">
-        <v>14.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="438">
@@ -15962,10 +15962,10 @@
         <v>114</v>
       </c>
       <c r="H443" s="3" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="I443" s="3" t="n">
-        <v>11.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="444">
@@ -16452,10 +16452,10 @@
         <v>324</v>
       </c>
       <c r="H457" s="4" t="n">
-        <v>10.8</v>
+        <v>4.5</v>
       </c>
       <c r="I457" s="4" t="n">
-        <v>64.8</v>
+        <v>27</v>
       </c>
     </row>
     <row r="458">
@@ -16487,10 +16487,10 @@
         <v>168</v>
       </c>
       <c r="H458" s="4" t="n">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I458" s="4" t="n">
-        <v>33.6</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="459">
@@ -16557,10 +16557,10 @@
         <v>48</v>
       </c>
       <c r="H460" s="4" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="I460" s="4" t="n">
-        <v>9.6</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="461">
@@ -16627,10 +16627,10 @@
         <v>42</v>
       </c>
       <c r="H462" s="3" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I462" s="3" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="463">
@@ -16697,10 +16697,10 @@
         <v>42</v>
       </c>
       <c r="H464" s="3" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="I464" s="3" t="n">
-        <v>7.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="465">
@@ -16732,10 +16732,10 @@
         <v>12</v>
       </c>
       <c r="H465" s="4" t="n">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="I465" s="4" t="n">
-        <v>12</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="466">
@@ -16802,10 +16802,10 @@
         <v>54</v>
       </c>
       <c r="H467" s="3" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="I467" s="3" t="n">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="468">
@@ -16837,10 +16837,10 @@
         <v>6</v>
       </c>
       <c r="H468" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I468" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="469">
@@ -16872,10 +16872,10 @@
         <v>282</v>
       </c>
       <c r="H469" s="4" t="n">
-        <v>5.2</v>
+        <v>3.9</v>
       </c>
       <c r="I469" s="4" t="n">
-        <v>31.2</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="470">
@@ -16942,10 +16942,10 @@
         <v>96</v>
       </c>
       <c r="H471" s="3" t="n">
-        <v>2.7</v>
+        <v>1.3</v>
       </c>
       <c r="I471" s="3" t="n">
-        <v>16.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="472">
@@ -17012,10 +17012,10 @@
         <v>66</v>
       </c>
       <c r="H473" s="4" t="n">
-        <v>2.2</v>
+        <v>0.9</v>
       </c>
       <c r="I473" s="4" t="n">
-        <v>13.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="474">
@@ -17047,10 +17047,10 @@
         <v>54</v>
       </c>
       <c r="H474" s="4" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="I474" s="4" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="475">
@@ -17082,10 +17082,10 @@
         <v>18</v>
       </c>
       <c r="H475" s="3" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="I475" s="3" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="476">
@@ -17117,10 +17117,10 @@
         <v>12</v>
       </c>
       <c r="H476" s="3" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I476" s="3" t="n">
-        <v>6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="477">
@@ -17222,10 +17222,10 @@
         <v>36</v>
       </c>
       <c r="H479" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="I479" s="3" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="480">
@@ -17257,10 +17257,10 @@
         <v>72</v>
       </c>
       <c r="H480" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="I480" s="3" t="n">
-        <v>14.4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="481">
@@ -17292,10 +17292,10 @@
         <v>36</v>
       </c>
       <c r="H481" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I481" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="482">
@@ -17362,10 +17362,10 @@
         <v>414</v>
       </c>
       <c r="H483" s="3" t="n">
-        <v>13.8</v>
+        <v>11.5</v>
       </c>
       <c r="I483" s="3" t="n">
-        <v>82.8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="484">
@@ -17397,10 +17397,10 @@
         <v>192</v>
       </c>
       <c r="H484" s="4" t="n">
-        <v>10.7</v>
+        <v>2.7</v>
       </c>
       <c r="I484" s="4" t="n">
-        <v>64.2</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="485">
@@ -17432,10 +17432,10 @@
         <v>120</v>
       </c>
       <c r="H485" s="4" t="n">
-        <v>10</v>
+        <v>3.3</v>
       </c>
       <c r="I485" s="4" t="n">
-        <v>60</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="486">
@@ -17467,10 +17467,10 @@
         <v>60</v>
       </c>
       <c r="H486" s="3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I486" s="3" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="487">
@@ -17502,10 +17502,10 @@
         <v>24</v>
       </c>
       <c r="H487" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I487" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="488">
@@ -17537,10 +17537,10 @@
         <v>30</v>
       </c>
       <c r="H488" s="4" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="I488" s="4" t="n">
-        <v>7.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="489">
@@ -17572,10 +17572,10 @@
         <v>42</v>
       </c>
       <c r="H489" s="4" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I489" s="4" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="490">
@@ -17607,10 +17607,10 @@
         <v>42</v>
       </c>
       <c r="H490" s="3" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="I490" s="3" t="n">
-        <v>6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="491">
@@ -17642,10 +17642,10 @@
         <v>24</v>
       </c>
       <c r="H491" s="3" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="I491" s="3" t="n">
-        <v>6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="492">
@@ -17677,10 +17677,10 @@
         <v>6</v>
       </c>
       <c r="H492" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I492" s="4" t="n">
-        <v>6</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Média mensal calculada entre primeira e última compra do ano por cliente/família
https://claude.ai/code/session_01SyvqAv69ozhh5ptHC31e4L
</commit_message>
<xml_diff>
--- a/relatorio_grao_por_vendedor.xlsx
+++ b/relatorio_grao_por_vendedor.xlsx
@@ -527,10 +527,10 @@
         <v>24</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.3</v>
+        <v>4</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -562,10 +562,10 @@
         <v>528</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>7.3</v>
+        <v>44</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>43.8</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>6</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -632,10 +632,10 @@
         <v>6</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -667,10 +667,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -737,10 +737,10 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -842,10 +842,10 @@
         <v>6</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -1157,10 +1157,10 @@
         <v>72</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="21">
@@ -1402,10 +1402,10 @@
         <v>24</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="28">
@@ -1437,10 +1437,10 @@
         <v>102</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>8.4</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="29">
@@ -1507,10 +1507,10 @@
         <v>60</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>10.2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -1542,10 +1542,10 @@
         <v>12</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32">
@@ -1577,10 +1577,10 @@
         <v>180</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33">
@@ -1647,10 +1647,10 @@
         <v>168</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>2.3</v>
+        <v>4</v>
       </c>
       <c r="I34" s="4" t="n">
-        <v>13.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="35">
@@ -1752,10 +1752,10 @@
         <v>84</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>7.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="38">
@@ -1892,10 +1892,10 @@
         <v>306</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>25.2</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="42">
@@ -1927,10 +1927,10 @@
         <v>150</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>25.2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43">
@@ -1997,10 +1997,10 @@
         <v>120</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>19.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45">
@@ -2172,10 +2172,10 @@
         <v>366</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>5.1</v>
+        <v>5.5</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>30.6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50">
@@ -2312,10 +2312,10 @@
         <v>84</v>
       </c>
       <c r="H53" s="4" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>7.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="54">
@@ -2382,10 +2382,10 @@
         <v>1278</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>17.8</v>
+        <v>19.4</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>106.8</v>
+        <v>116.4</v>
       </c>
     </row>
     <row r="56">
@@ -2417,10 +2417,10 @@
         <v>510</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>14.2</v>
+        <v>17</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>85.2</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57">
@@ -2452,10 +2452,10 @@
         <v>6</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
@@ -2557,10 +2557,10 @@
         <v>120</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="I60" s="4" t="n">
-        <v>10.2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="61">
@@ -2627,10 +2627,10 @@
         <v>372</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>31.2</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="63">
@@ -2697,10 +2697,10 @@
         <v>12</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
@@ -2732,10 +2732,10 @@
         <v>12</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66">
@@ -2767,10 +2767,10 @@
         <v>24</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="67">
@@ -2802,10 +2802,10 @@
         <v>420</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>5.8</v>
+        <v>35</v>
       </c>
       <c r="I67" s="4" t="n">
-        <v>34.8</v>
+        <v>210</v>
       </c>
     </row>
     <row r="68">
@@ -2942,10 +2942,10 @@
         <v>24</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I71" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="72">
@@ -2977,10 +2977,10 @@
         <v>12</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I72" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73">
@@ -3082,10 +3082,10 @@
         <v>66</v>
       </c>
       <c r="H75" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I75" s="4" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -3152,10 +3152,10 @@
         <v>48</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="78">
@@ -3187,10 +3187,10 @@
         <v>12</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="79">
@@ -3327,10 +3327,10 @@
         <v>54</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="I82" s="3" t="n">
-        <v>9</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="83">
@@ -3397,10 +3397,10 @@
         <v>24</v>
       </c>
       <c r="H84" s="4" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I84" s="4" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="85">
@@ -3432,10 +3432,10 @@
         <v>48</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="86">
@@ -3467,10 +3467,10 @@
         <v>24</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87">
@@ -3677,10 +3677,10 @@
         <v>18</v>
       </c>
       <c r="H92" s="4" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I92" s="4" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="93">
@@ -3817,10 +3817,10 @@
         <v>72</v>
       </c>
       <c r="H96" s="4" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="I96" s="4" t="n">
-        <v>12</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="97">
@@ -4097,10 +4097,10 @@
         <v>18</v>
       </c>
       <c r="H104" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I104" s="4" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="105">
@@ -4132,10 +4132,10 @@
         <v>168</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="I105" s="3" t="n">
-        <v>13.8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="106">
@@ -4167,10 +4167,10 @@
         <v>72</v>
       </c>
       <c r="H106" s="3" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="I106" s="3" t="n">
-        <v>12</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="107">
@@ -4202,10 +4202,10 @@
         <v>18</v>
       </c>
       <c r="H107" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I107" s="4" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="108">
@@ -4237,10 +4237,10 @@
         <v>6</v>
       </c>
       <c r="H108" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I108" s="4" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="109">
@@ -4307,10 +4307,10 @@
         <v>234</v>
       </c>
       <c r="H110" s="3" t="n">
-        <v>6.5</v>
+        <v>7.8</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>39</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="111">
@@ -4377,10 +4377,10 @@
         <v>6</v>
       </c>
       <c r="H112" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I112" s="4" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="113">
@@ -4412,10 +4412,10 @@
         <v>30</v>
       </c>
       <c r="H113" s="3" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
       <c r="I113" s="3" t="n">
-        <v>2.4</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="114">
@@ -4447,10 +4447,10 @@
         <v>252</v>
       </c>
       <c r="H114" s="4" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="I114" s="4" t="n">
-        <v>21</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="115">
@@ -4587,10 +4587,10 @@
         <v>18</v>
       </c>
       <c r="H118" s="4" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="I118" s="4" t="n">
-        <v>1.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="119">
@@ -4797,10 +4797,10 @@
         <v>42</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="I124" s="3" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="125">
@@ -4832,10 +4832,10 @@
         <v>54</v>
       </c>
       <c r="H125" s="4" t="n">
-        <v>0.8</v>
+        <v>3</v>
       </c>
       <c r="I125" s="4" t="n">
-        <v>4.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126">
@@ -4867,10 +4867,10 @@
         <v>90</v>
       </c>
       <c r="H126" s="4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I126" s="4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="127">
@@ -4937,10 +4937,10 @@
         <v>12</v>
       </c>
       <c r="H128" s="4" t="n">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="I128" s="4" t="n">
-        <v>1.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="129">
@@ -4972,10 +4972,10 @@
         <v>18</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>0.2</v>
+        <v>3</v>
       </c>
       <c r="I129" s="3" t="n">
-        <v>1.2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="130">
@@ -5007,10 +5007,10 @@
         <v>96</v>
       </c>
       <c r="H130" s="4" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="I130" s="4" t="n">
-        <v>7.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="131">
@@ -5112,10 +5112,10 @@
         <v>198</v>
       </c>
       <c r="H133" s="4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="I133" s="4" t="n">
-        <v>16.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="134">
@@ -5217,10 +5217,10 @@
         <v>60</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="I136" s="3" t="n">
-        <v>10.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="137">
@@ -5252,10 +5252,10 @@
         <v>54</v>
       </c>
       <c r="H137" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I137" s="4" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="138">
@@ -5287,10 +5287,10 @@
         <v>24</v>
       </c>
       <c r="H138" s="4" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I138" s="4" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="139">
@@ -5322,10 +5322,10 @@
         <v>30</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I139" s="3" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="140">
@@ -5357,10 +5357,10 @@
         <v>12</v>
       </c>
       <c r="H140" s="3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I140" s="3" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="141">
@@ -5392,10 +5392,10 @@
         <v>6</v>
       </c>
       <c r="H141" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I141" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="142">
@@ -5427,10 +5427,10 @@
         <v>48</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I142" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="143">
@@ -5462,10 +5462,10 @@
         <v>18</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I143" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="144">
@@ -5497,10 +5497,10 @@
         <v>54</v>
       </c>
       <c r="H144" s="4" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="I144" s="4" t="n">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="145">
@@ -5567,10 +5567,10 @@
         <v>6</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I146" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="147">
@@ -5602,10 +5602,10 @@
         <v>42</v>
       </c>
       <c r="H147" s="4" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I147" s="4" t="n">
-        <v>3.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="148">
@@ -5637,10 +5637,10 @@
         <v>24</v>
       </c>
       <c r="H148" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I148" s="4" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="149">
@@ -5672,10 +5672,10 @@
         <v>12</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="150">
@@ -5707,10 +5707,10 @@
         <v>30</v>
       </c>
       <c r="H150" s="4" t="n">
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="I150" s="4" t="n">
-        <v>4.8</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="151">
@@ -5742,10 +5742,10 @@
         <v>6</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I151" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="152">
@@ -5777,10 +5777,10 @@
         <v>24</v>
       </c>
       <c r="H152" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I152" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="153">
@@ -5847,10 +5847,10 @@
         <v>24</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I154" s="3" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155">
@@ -5882,10 +5882,10 @@
         <v>6</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I155" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="156">
@@ -5952,10 +5952,10 @@
         <v>18</v>
       </c>
       <c r="H157" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I157" s="4" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="158">
@@ -5987,10 +5987,10 @@
         <v>12</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I158" s="3" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="159">
@@ -6022,10 +6022,10 @@
         <v>24</v>
       </c>
       <c r="H159" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I159" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="160">
@@ -6057,10 +6057,10 @@
         <v>12</v>
       </c>
       <c r="H160" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I160" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="161">
@@ -6127,10 +6127,10 @@
         <v>66</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="I162" s="3" t="n">
-        <v>10.8</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="163">
@@ -6162,10 +6162,10 @@
         <v>24</v>
       </c>
       <c r="H163" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I163" s="4" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="164">
@@ -6197,10 +6197,10 @@
         <v>12</v>
       </c>
       <c r="H164" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I164" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="165">
@@ -6267,10 +6267,10 @@
         <v>24</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I166" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="167">
@@ -6302,10 +6302,10 @@
         <v>30</v>
       </c>
       <c r="H167" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="I167" s="4" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="168">
@@ -6337,10 +6337,10 @@
         <v>18</v>
       </c>
       <c r="H168" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I168" s="4" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="169">
@@ -6477,10 +6477,10 @@
         <v>18</v>
       </c>
       <c r="H172" s="4" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I172" s="4" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="173">
@@ -6687,10 +6687,10 @@
         <v>30</v>
       </c>
       <c r="H178" s="3" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I178" s="3" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="179">
@@ -6757,10 +6757,10 @@
         <v>54</v>
       </c>
       <c r="H180" s="4" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="I180" s="4" t="n">
-        <v>9</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="181">
@@ -6932,10 +6932,10 @@
         <v>90</v>
       </c>
       <c r="H185" s="3" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="I185" s="3" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="186">
@@ -6967,10 +6967,10 @@
         <v>24</v>
       </c>
       <c r="H186" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I186" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="187">
@@ -7002,10 +7002,10 @@
         <v>60</v>
       </c>
       <c r="H187" s="4" t="n">
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="I187" s="4" t="n">
-        <v>4.8</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="188">
@@ -7037,10 +7037,10 @@
         <v>24</v>
       </c>
       <c r="H188" s="4" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I188" s="4" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="189">
@@ -7177,10 +7177,10 @@
         <v>6</v>
       </c>
       <c r="H192" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I192" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="193">
@@ -7212,10 +7212,10 @@
         <v>30</v>
       </c>
       <c r="H193" s="4" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="I193" s="4" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="194">
@@ -7422,10 +7422,10 @@
         <v>18</v>
       </c>
       <c r="H199" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I199" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="200">
@@ -7457,10 +7457,10 @@
         <v>48</v>
       </c>
       <c r="H200" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I200" s="4" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="201">
@@ -7492,10 +7492,10 @@
         <v>24</v>
       </c>
       <c r="H201" s="4" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I201" s="4" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="202">
@@ -7527,10 +7527,10 @@
         <v>18</v>
       </c>
       <c r="H202" s="3" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I202" s="3" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="203">
@@ -7562,10 +7562,10 @@
         <v>12</v>
       </c>
       <c r="H203" s="3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I203" s="3" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="204">
@@ -7702,10 +7702,10 @@
         <v>180</v>
       </c>
       <c r="H207" s="4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I207" s="4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="208">
@@ -7737,10 +7737,10 @@
         <v>54</v>
       </c>
       <c r="H208" s="4" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="I208" s="4" t="n">
-        <v>9</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="209">
@@ -7842,10 +7842,10 @@
         <v>42</v>
       </c>
       <c r="H211" s="4" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="I211" s="4" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="212">
@@ -7877,10 +7877,10 @@
         <v>24</v>
       </c>
       <c r="H212" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I212" s="4" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="213">
@@ -7912,10 +7912,10 @@
         <v>24</v>
       </c>
       <c r="H213" s="3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="I213" s="3" t="n">
-        <v>1.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="214">
@@ -7947,10 +7947,10 @@
         <v>180</v>
       </c>
       <c r="H214" s="4" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="I214" s="4" t="n">
-        <v>15</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="215">
@@ -8052,10 +8052,10 @@
         <v>66</v>
       </c>
       <c r="H217" s="3" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="I217" s="3" t="n">
-        <v>10.8</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="218">
@@ -8192,10 +8192,10 @@
         <v>48</v>
       </c>
       <c r="H221" s="3" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="I221" s="3" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="222">
@@ -8297,10 +8297,10 @@
         <v>348</v>
       </c>
       <c r="H224" s="3" t="n">
-        <v>4.8</v>
+        <v>29</v>
       </c>
       <c r="I224" s="3" t="n">
-        <v>28.8</v>
+        <v>174</v>
       </c>
     </row>
     <row r="225">
@@ -8332,10 +8332,10 @@
         <v>48</v>
       </c>
       <c r="H225" s="4" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="I225" s="4" t="n">
-        <v>4.2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="226">
@@ -8367,10 +8367,10 @@
         <v>270</v>
       </c>
       <c r="H226" s="3" t="n">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="I226" s="3" t="n">
-        <v>22.8</v>
+        <v>27</v>
       </c>
     </row>
     <row r="227">
@@ -8437,10 +8437,10 @@
         <v>324</v>
       </c>
       <c r="H228" s="4" t="n">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="I228" s="4" t="n">
-        <v>27</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="229">
@@ -8507,10 +8507,10 @@
         <v>168</v>
       </c>
       <c r="H230" s="3" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="I230" s="3" t="n">
-        <v>13.8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231">
@@ -8647,10 +8647,10 @@
         <v>120</v>
       </c>
       <c r="H234" s="3" t="n">
-        <v>1.7</v>
+        <v>2.2</v>
       </c>
       <c r="I234" s="3" t="n">
-        <v>10.2</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="235">
@@ -8682,10 +8682,10 @@
         <v>60</v>
       </c>
       <c r="H235" s="3" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="I235" s="3" t="n">
-        <v>10.2</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="236">
@@ -8822,10 +8822,10 @@
         <v>72</v>
       </c>
       <c r="H239" s="3" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="I239" s="3" t="n">
-        <v>12</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="240">
@@ -8857,10 +8857,10 @@
         <v>258</v>
       </c>
       <c r="H240" s="4" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="I240" s="4" t="n">
-        <v>21.6</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="241">
@@ -8927,10 +8927,10 @@
         <v>264</v>
       </c>
       <c r="H242" s="3" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="I242" s="3" t="n">
-        <v>22.2</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="243">
@@ -8997,10 +8997,10 @@
         <v>600</v>
       </c>
       <c r="H244" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="I244" s="4" t="n">
-        <v>49.8</v>
+        <v>60</v>
       </c>
     </row>
     <row r="245">
@@ -9032,10 +9032,10 @@
         <v>150</v>
       </c>
       <c r="H245" s="4" t="n">
-        <v>4.2</v>
+        <v>25</v>
       </c>
       <c r="I245" s="4" t="n">
-        <v>25.2</v>
+        <v>150</v>
       </c>
     </row>
     <row r="246">
@@ -9067,10 +9067,10 @@
         <v>12</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="I246" s="3" t="n">
-        <v>1.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="247">
@@ -9102,10 +9102,10 @@
         <v>30</v>
       </c>
       <c r="H247" s="4" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="I247" s="4" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="248">
@@ -9172,10 +9172,10 @@
         <v>12</v>
       </c>
       <c r="H249" s="3" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="I249" s="3" t="n">
-        <v>1.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="250">
@@ -9207,10 +9207,10 @@
         <v>18</v>
       </c>
       <c r="H250" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I250" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="251">
@@ -9242,10 +9242,10 @@
         <v>6</v>
       </c>
       <c r="H251" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I251" s="4" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="252">
@@ -9277,10 +9277,10 @@
         <v>438</v>
       </c>
       <c r="H252" s="3" t="n">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I252" s="3" t="n">
-        <v>36.6</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="253">
@@ -9382,10 +9382,10 @@
         <v>24</v>
       </c>
       <c r="H255" s="4" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I255" s="4" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="256">
@@ -9487,10 +9487,10 @@
         <v>84</v>
       </c>
       <c r="H258" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="I258" s="4" t="n">
-        <v>7.2</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="259">
@@ -9522,10 +9522,10 @@
         <v>36</v>
       </c>
       <c r="H259" s="3" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I259" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="260">
@@ -9592,10 +9592,10 @@
         <v>12</v>
       </c>
       <c r="H261" s="4" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="I261" s="4" t="n">
-        <v>1.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="262">
@@ -9627,10 +9627,10 @@
         <v>12</v>
       </c>
       <c r="H262" s="4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I262" s="4" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="263">
@@ -9662,10 +9662,10 @@
         <v>30</v>
       </c>
       <c r="H263" s="3" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="I263" s="3" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="264">
@@ -9697,10 +9697,10 @@
         <v>24</v>
       </c>
       <c r="H264" s="3" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I264" s="3" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="265">
@@ -9732,10 +9732,10 @@
         <v>66</v>
       </c>
       <c r="H265" s="4" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="I265" s="4" t="n">
-        <v>5.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="266">
@@ -9837,10 +9837,10 @@
         <v>42</v>
       </c>
       <c r="H268" s="3" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="I268" s="3" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="269">
@@ -9872,10 +9872,10 @@
         <v>30</v>
       </c>
       <c r="H269" s="4" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="I269" s="4" t="n">
-        <v>4.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="270">
@@ -9907,10 +9907,10 @@
         <v>24</v>
       </c>
       <c r="H270" s="3" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="I270" s="3" t="n">
-        <v>4.2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="271">
@@ -10327,10 +10327,10 @@
         <v>108</v>
       </c>
       <c r="H282" s="4" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="I282" s="4" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="283">
@@ -10362,10 +10362,10 @@
         <v>48</v>
       </c>
       <c r="H283" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I283" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="284">
@@ -10397,10 +10397,10 @@
         <v>48</v>
       </c>
       <c r="H284" s="4" t="n">
-        <v>0.7</v>
+        <v>2.7</v>
       </c>
       <c r="I284" s="4" t="n">
-        <v>4.2</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="285">
@@ -10642,10 +10642,10 @@
         <v>60</v>
       </c>
       <c r="H291" s="3" t="n">
-        <v>1.7</v>
+        <v>5</v>
       </c>
       <c r="I291" s="3" t="n">
-        <v>10.2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="292">
@@ -10677,10 +10677,10 @@
         <v>126</v>
       </c>
       <c r="H292" s="3" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="I292" s="3" t="n">
-        <v>21</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="293">
@@ -10782,10 +10782,10 @@
         <v>66</v>
       </c>
       <c r="H295" s="3" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="I295" s="3" t="n">
-        <v>5.4</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="296">
@@ -10922,10 +10922,10 @@
         <v>30</v>
       </c>
       <c r="H299" s="3" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="I299" s="3" t="n">
-        <v>4.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="300">
@@ -11377,10 +11377,10 @@
         <v>3168</v>
       </c>
       <c r="H312" s="4" t="n">
-        <v>44</v>
+        <v>52.8</v>
       </c>
       <c r="I312" s="4" t="n">
-        <v>264</v>
+        <v>316.8</v>
       </c>
     </row>
     <row r="313">
@@ -11412,10 +11412,10 @@
         <v>882</v>
       </c>
       <c r="H313" s="4" t="n">
-        <v>24.5</v>
+        <v>29.4</v>
       </c>
       <c r="I313" s="4" t="n">
-        <v>147</v>
+        <v>176.4</v>
       </c>
     </row>
     <row r="314">
@@ -11517,10 +11517,10 @@
         <v>132</v>
       </c>
       <c r="H316" s="4" t="n">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="I316" s="4" t="n">
-        <v>22.2</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="317">
@@ -11587,10 +11587,10 @@
         <v>36</v>
       </c>
       <c r="H318" s="3" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="I318" s="3" t="n">
-        <v>6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="319">
@@ -11867,10 +11867,10 @@
         <v>108</v>
       </c>
       <c r="H326" s="4" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="I326" s="4" t="n">
-        <v>9</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="327">
@@ -11902,10 +11902,10 @@
         <v>12</v>
       </c>
       <c r="H327" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I327" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="328">
@@ -11937,10 +11937,10 @@
         <v>420</v>
       </c>
       <c r="H328" s="4" t="n">
-        <v>5.8</v>
+        <v>7.8</v>
       </c>
       <c r="I328" s="4" t="n">
-        <v>34.8</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="329">
@@ -12007,10 +12007,10 @@
         <v>24</v>
       </c>
       <c r="H330" s="3" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I330" s="3" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="331">
@@ -12077,10 +12077,10 @@
         <v>6</v>
       </c>
       <c r="H332" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I332" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="333">
@@ -12112,10 +12112,10 @@
         <v>24</v>
       </c>
       <c r="H333" s="3" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="I333" s="3" t="n">
-        <v>4.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="334">
@@ -12147,10 +12147,10 @@
         <v>24</v>
       </c>
       <c r="H334" s="3" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="I334" s="3" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="335">
@@ -12182,10 +12182,10 @@
         <v>24</v>
       </c>
       <c r="H335" s="4" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I335" s="4" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="336">
@@ -12217,10 +12217,10 @@
         <v>66</v>
       </c>
       <c r="H336" s="3" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I336" s="3" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="337">
@@ -12252,10 +12252,10 @@
         <v>24</v>
       </c>
       <c r="H337" s="3" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="I337" s="3" t="n">
-        <v>4.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="338">
@@ -12287,10 +12287,10 @@
         <v>60</v>
       </c>
       <c r="H338" s="4" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I338" s="4" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="339">
@@ -12357,10 +12357,10 @@
         <v>6</v>
       </c>
       <c r="H340" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I340" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="341">
@@ -12427,10 +12427,10 @@
         <v>18</v>
       </c>
       <c r="H342" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I342" s="4" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="343">
@@ -12742,10 +12742,10 @@
         <v>186</v>
       </c>
       <c r="H351" s="3" t="n">
-        <v>2.6</v>
+        <v>5.2</v>
       </c>
       <c r="I351" s="3" t="n">
-        <v>15.6</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="352">
@@ -12777,10 +12777,10 @@
         <v>150</v>
       </c>
       <c r="H352" s="3" t="n">
-        <v>2.1</v>
+        <v>4.2</v>
       </c>
       <c r="I352" s="3" t="n">
-        <v>12.6</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="353">
@@ -12882,10 +12882,10 @@
         <v>30</v>
       </c>
       <c r="H355" s="4" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="I355" s="4" t="n">
-        <v>4.8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="356">
@@ -12987,10 +12987,10 @@
         <v>120</v>
       </c>
       <c r="H358" s="4" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="I358" s="4" t="n">
-        <v>10.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="359">
@@ -13022,10 +13022,10 @@
         <v>30</v>
       </c>
       <c r="H359" s="4" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="I359" s="4" t="n">
-        <v>4.8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="360">
@@ -13267,10 +13267,10 @@
         <v>96</v>
       </c>
       <c r="H366" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="I366" s="4" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="367">
@@ -13372,10 +13372,10 @@
         <v>36</v>
       </c>
       <c r="H369" s="4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="I369" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="370">
@@ -13582,10 +13582,10 @@
         <v>84</v>
       </c>
       <c r="H375" s="3" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="I375" s="3" t="n">
-        <v>13.8</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="376">
@@ -13617,10 +13617,10 @@
         <v>6</v>
       </c>
       <c r="H376" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I376" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="377">
@@ -13722,10 +13722,10 @@
         <v>90</v>
       </c>
       <c r="H379" s="4" t="n">
-        <v>1.2</v>
+        <v>2.5</v>
       </c>
       <c r="I379" s="4" t="n">
-        <v>7.2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="380">
@@ -13757,10 +13757,10 @@
         <v>330</v>
       </c>
       <c r="H380" s="3" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="I380" s="3" t="n">
-        <v>27.6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="381">
@@ -13792,10 +13792,10 @@
         <v>150</v>
       </c>
       <c r="H381" s="3" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="I381" s="3" t="n">
-        <v>25.2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="382">
@@ -13862,10 +13862,10 @@
         <v>204</v>
       </c>
       <c r="H383" s="4" t="n">
-        <v>5.7</v>
+        <v>6.8</v>
       </c>
       <c r="I383" s="4" t="n">
-        <v>34.2</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="384">
@@ -13897,10 +13897,10 @@
         <v>24</v>
       </c>
       <c r="H384" s="3" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I384" s="3" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="385">
@@ -14037,10 +14037,10 @@
         <v>102</v>
       </c>
       <c r="H388" s="3" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="I388" s="3" t="n">
-        <v>16.8</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="389">
@@ -14072,10 +14072,10 @@
         <v>66</v>
       </c>
       <c r="H389" s="4" t="n">
-        <v>0.9</v>
+        <v>2.2</v>
       </c>
       <c r="I389" s="4" t="n">
-        <v>5.4</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="390">
@@ -14142,10 +14142,10 @@
         <v>72</v>
       </c>
       <c r="H391" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I391" s="3" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="392">
@@ -14247,10 +14247,10 @@
         <v>6</v>
       </c>
       <c r="H394" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I394" s="3" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="395">
@@ -14282,10 +14282,10 @@
         <v>96</v>
       </c>
       <c r="H395" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="I395" s="4" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="396">
@@ -14317,10 +14317,10 @@
         <v>6</v>
       </c>
       <c r="H396" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I396" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="397">
@@ -14352,10 +14352,10 @@
         <v>84</v>
       </c>
       <c r="H397" s="3" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="I397" s="3" t="n">
-        <v>7.2</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="398">
@@ -14387,10 +14387,10 @@
         <v>42</v>
       </c>
       <c r="H398" s="3" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="I398" s="3" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="399">
@@ -14422,10 +14422,10 @@
         <v>24</v>
       </c>
       <c r="H399" s="4" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="I399" s="4" t="n">
-        <v>1.8</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="400">
@@ -14457,10 +14457,10 @@
         <v>30</v>
       </c>
       <c r="H400" s="3" t="n">
-        <v>0.4</v>
+        <v>5</v>
       </c>
       <c r="I400" s="3" t="n">
-        <v>2.4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="401">
@@ -14492,10 +14492,10 @@
         <v>78</v>
       </c>
       <c r="H401" s="4" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="I401" s="4" t="n">
-        <v>6.6</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="402">
@@ -14562,10 +14562,10 @@
         <v>12</v>
       </c>
       <c r="H403" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I403" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="404">
@@ -14597,10 +14597,10 @@
         <v>18</v>
       </c>
       <c r="H404" s="3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I404" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="405">
@@ -14667,10 +14667,10 @@
         <v>102</v>
       </c>
       <c r="H406" s="3" t="n">
-        <v>2.8</v>
+        <v>5.7</v>
       </c>
       <c r="I406" s="3" t="n">
-        <v>16.8</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="407">
@@ -14702,10 +14702,10 @@
         <v>12</v>
       </c>
       <c r="H407" s="4" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I407" s="4" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="408">
@@ -14737,10 +14737,10 @@
         <v>18</v>
       </c>
       <c r="H408" s="3" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="I408" s="3" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="409">
@@ -14772,10 +14772,10 @@
         <v>18</v>
       </c>
       <c r="H409" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I409" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="410">
@@ -14807,10 +14807,10 @@
         <v>6</v>
       </c>
       <c r="H410" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I410" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="411">
@@ -14842,10 +14842,10 @@
         <v>90</v>
       </c>
       <c r="H411" s="3" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="I411" s="3" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="412">
@@ -14877,10 +14877,10 @@
         <v>30</v>
       </c>
       <c r="H412" s="3" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I412" s="3" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="413">
@@ -14947,10 +14947,10 @@
         <v>48</v>
       </c>
       <c r="H414" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="I414" s="4" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="415">
@@ -15157,10 +15157,10 @@
         <v>30</v>
       </c>
       <c r="H420" s="3" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="I420" s="3" t="n">
-        <v>4.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="421">
@@ -15262,10 +15262,10 @@
         <v>30</v>
       </c>
       <c r="H423" s="3" t="n">
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="I423" s="3" t="n">
-        <v>4.8</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="424">
@@ -15297,10 +15297,10 @@
         <v>66</v>
       </c>
       <c r="H424" s="3" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="I424" s="3" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="425">
@@ -15332,10 +15332,10 @@
         <v>24</v>
       </c>
       <c r="H425" s="3" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="I425" s="3" t="n">
-        <v>4.2</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="426">
@@ -15472,10 +15472,10 @@
         <v>12</v>
       </c>
       <c r="H429" s="3" t="n">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="I429" s="3" t="n">
-        <v>1.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="430">
@@ -15682,10 +15682,10 @@
         <v>30</v>
       </c>
       <c r="H435" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I435" s="4" t="n">
-        <v>4.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="436">
@@ -15752,10 +15752,10 @@
         <v>72</v>
       </c>
       <c r="H437" s="3" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="I437" s="3" t="n">
-        <v>12</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="438">
@@ -15962,10 +15962,10 @@
         <v>114</v>
       </c>
       <c r="H443" s="3" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="I443" s="3" t="n">
-        <v>9.6</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="444">
@@ -16452,10 +16452,10 @@
         <v>324</v>
       </c>
       <c r="H457" s="4" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="I457" s="4" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="458">
@@ -16487,10 +16487,10 @@
         <v>168</v>
       </c>
       <c r="H458" s="4" t="n">
-        <v>4.7</v>
+        <v>5.6</v>
       </c>
       <c r="I458" s="4" t="n">
-        <v>28.2</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="459">
@@ -16557,10 +16557,10 @@
         <v>48</v>
       </c>
       <c r="H460" s="4" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="I460" s="4" t="n">
-        <v>7.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="461">
@@ -16732,10 +16732,10 @@
         <v>12</v>
       </c>
       <c r="H465" s="4" t="n">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="I465" s="4" t="n">
-        <v>1.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="466">
@@ -16802,10 +16802,10 @@
         <v>54</v>
       </c>
       <c r="H467" s="3" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I467" s="3" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="468">
@@ -16837,10 +16837,10 @@
         <v>6</v>
       </c>
       <c r="H468" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I468" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="469">
@@ -16872,10 +16872,10 @@
         <v>282</v>
       </c>
       <c r="H469" s="4" t="n">
-        <v>3.9</v>
+        <v>5.2</v>
       </c>
       <c r="I469" s="4" t="n">
-        <v>23.4</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="470">
@@ -16942,10 +16942,10 @@
         <v>96</v>
       </c>
       <c r="H471" s="3" t="n">
-        <v>1.3</v>
+        <v>2.7</v>
       </c>
       <c r="I471" s="3" t="n">
-        <v>7.8</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="472">
@@ -17012,10 +17012,10 @@
         <v>66</v>
       </c>
       <c r="H473" s="4" t="n">
-        <v>0.9</v>
+        <v>2.2</v>
       </c>
       <c r="I473" s="4" t="n">
-        <v>5.4</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="474">
@@ -17047,10 +17047,10 @@
         <v>54</v>
       </c>
       <c r="H474" s="4" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="I474" s="4" t="n">
-        <v>9</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="475">
@@ -17082,10 +17082,10 @@
         <v>18</v>
       </c>
       <c r="H475" s="3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I475" s="3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="476">
@@ -17117,10 +17117,10 @@
         <v>12</v>
       </c>
       <c r="H476" s="3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="I476" s="3" t="n">
-        <v>1.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="477">
@@ -17222,10 +17222,10 @@
         <v>36</v>
       </c>
       <c r="H479" s="3" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="I479" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="480">
@@ -17292,10 +17292,10 @@
         <v>36</v>
       </c>
       <c r="H481" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I481" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="482">
@@ -17362,10 +17362,10 @@
         <v>414</v>
       </c>
       <c r="H483" s="3" t="n">
-        <v>11.5</v>
+        <v>13.8</v>
       </c>
       <c r="I483" s="3" t="n">
-        <v>69</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="484">
@@ -17397,10 +17397,10 @@
         <v>192</v>
       </c>
       <c r="H484" s="4" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="I484" s="4" t="n">
-        <v>16.2</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="485">
@@ -17432,10 +17432,10 @@
         <v>120</v>
       </c>
       <c r="H485" s="4" t="n">
-        <v>3.3</v>
+        <v>6.7</v>
       </c>
       <c r="I485" s="4" t="n">
-        <v>19.8</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="486">
@@ -17467,10 +17467,10 @@
         <v>60</v>
       </c>
       <c r="H486" s="3" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I486" s="3" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="487">
@@ -17502,10 +17502,10 @@
         <v>24</v>
       </c>
       <c r="H487" s="3" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I487" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="488">
@@ -17537,10 +17537,10 @@
         <v>30</v>
       </c>
       <c r="H488" s="4" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="I488" s="4" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="489">
@@ -17572,10 +17572,10 @@
         <v>42</v>
       </c>
       <c r="H489" s="4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="I489" s="4" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="490">
@@ -17677,10 +17677,10 @@
         <v>6</v>
       </c>
       <c r="H492" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I492" s="4" t="n">
-        <v>0.6</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrigir média para clientes com uma única compra (divisor mínimo = 1 mês)
https://claude.ai/code/session_01SyvqAv69ozhh5ptHC31e4L
</commit_message>
<xml_diff>
--- a/relatorio_grao_por_vendedor.xlsx
+++ b/relatorio_grao_por_vendedor.xlsx
@@ -527,10 +527,10 @@
         <v>24</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>121.8</v>
+        <v>4</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>730.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -562,10 +562,10 @@
         <v>528</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>95.7</v>
+        <v>88</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>574.2</v>
+        <v>528</v>
       </c>
     </row>
     <row r="4">
@@ -597,10 +597,10 @@
         <v>6</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -632,10 +632,10 @@
         <v>6</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -667,10 +667,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -807,10 +807,10 @@
         <v>6</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -2382,10 +2382,10 @@
         <v>6</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56">
@@ -2662,10 +2662,10 @@
         <v>12</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64">
@@ -4167,10 +4167,10 @@
         <v>6</v>
       </c>
       <c r="H106" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I106" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107">
@@ -4307,10 +4307,10 @@
         <v>6</v>
       </c>
       <c r="H110" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I110" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111">
@@ -4867,10 +4867,10 @@
         <v>12</v>
       </c>
       <c r="H126" s="4" t="n">
-        <v>10.1</v>
+        <v>2</v>
       </c>
       <c r="I126" s="4" t="n">
-        <v>60.6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="127">
@@ -4902,10 +4902,10 @@
         <v>18</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="I127" s="3" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
     </row>
     <row r="128">
@@ -5322,10 +5322,10 @@
         <v>6</v>
       </c>
       <c r="H139" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I139" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="140">
@@ -5497,10 +5497,10 @@
         <v>6</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I144" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="145">
@@ -5672,10 +5672,10 @@
         <v>6</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="150">
@@ -5812,10 +5812,10 @@
         <v>6</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I153" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="154">
@@ -7072,10 +7072,10 @@
         <v>6</v>
       </c>
       <c r="H189" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I189" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="190">
@@ -8227,10 +8227,10 @@
         <v>48</v>
       </c>
       <c r="H222" s="4" t="n">
-        <v>14.3</v>
+        <v>8</v>
       </c>
       <c r="I222" s="4" t="n">
-        <v>85.8</v>
+        <v>48</v>
       </c>
     </row>
     <row r="223">
@@ -8927,10 +8927,10 @@
         <v>150</v>
       </c>
       <c r="H242" s="4" t="n">
-        <v>761</v>
+        <v>25</v>
       </c>
       <c r="I242" s="4" t="n">
-        <v>4566</v>
+        <v>150</v>
       </c>
     </row>
     <row r="243">
@@ -9067,10 +9067,10 @@
         <v>12</v>
       </c>
       <c r="H246" s="3" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="I246" s="3" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="247">
@@ -9137,10 +9137,10 @@
         <v>6</v>
       </c>
       <c r="H248" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I248" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="249">
@@ -9802,10 +9802,10 @@
         <v>24</v>
       </c>
       <c r="H267" s="3" t="n">
-        <v>12.2</v>
+        <v>4</v>
       </c>
       <c r="I267" s="3" t="n">
-        <v>73.2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="268">
@@ -11937,10 +11937,10 @@
         <v>6</v>
       </c>
       <c r="H328" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I328" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="329">
@@ -12217,10 +12217,10 @@
         <v>6</v>
       </c>
       <c r="H336" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I336" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="337">
@@ -12847,10 +12847,10 @@
         <v>30</v>
       </c>
       <c r="H354" s="4" t="n">
-        <v>152.2</v>
+        <v>5</v>
       </c>
       <c r="I354" s="4" t="n">
-        <v>913.2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="355">
@@ -13442,10 +13442,10 @@
         <v>6</v>
       </c>
       <c r="H371" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I371" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="372">
@@ -14072,10 +14072,10 @@
         <v>6</v>
       </c>
       <c r="H389" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I389" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="390">
@@ -14247,10 +14247,10 @@
         <v>30</v>
       </c>
       <c r="H394" s="3" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="I394" s="3" t="n">
-        <v>32.4</v>
+        <v>30</v>
       </c>
     </row>
     <row r="395">
@@ -14492,10 +14492,10 @@
         <v>12</v>
       </c>
       <c r="H401" s="4" t="n">
-        <v>10.1</v>
+        <v>2</v>
       </c>
       <c r="I401" s="4" t="n">
-        <v>60.6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="402">
@@ -14527,10 +14527,10 @@
         <v>18</v>
       </c>
       <c r="H402" s="3" t="n">
-        <v>4.3</v>
+        <v>3</v>
       </c>
       <c r="I402" s="3" t="n">
-        <v>25.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="403">
@@ -14597,10 +14597,10 @@
         <v>6</v>
       </c>
       <c r="H404" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I404" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="405">
@@ -15262,10 +15262,10 @@
         <v>12</v>
       </c>
       <c r="H423" s="3" t="n">
-        <v>4.3</v>
+        <v>2</v>
       </c>
       <c r="I423" s="3" t="n">
-        <v>25.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="424">
@@ -16522,10 +16522,10 @@
         <v>12</v>
       </c>
       <c r="H459" s="4" t="n">
-        <v>4.3</v>
+        <v>2</v>
       </c>
       <c r="I459" s="4" t="n">
-        <v>25.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="460">
@@ -16627,10 +16627,10 @@
         <v>6</v>
       </c>
       <c r="H462" s="3" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I462" s="3" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="463">
@@ -17467,10 +17467,10 @@
         <v>6</v>
       </c>
       <c r="H486" s="4" t="n">
-        <v>30.4</v>
+        <v>1</v>
       </c>
       <c r="I486" s="4" t="n">
-        <v>182.4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>